<commit_message>
zmiany w pliku ryzyko.xlsx
</commit_message>
<xml_diff>
--- a/Ryzyko.xlsx
+++ b/Ryzyko.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\owcza\Desktop\nw\inzynieria-oprogramowania\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6429108-176F-4246-BDDA-630D635DBD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39264F62-3CFB-4753-B417-FC658910245C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="24">
   <si>
     <t>1. Poniżej wpiszcie numer indeksu i imię i nazwisko poszczególnych osób w zespole</t>
   </si>
@@ -564,6 +564,12 @@
       <c r="B13" t="s">
         <v>21</v>
       </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
@@ -572,6 +578,12 @@
       <c r="B14" t="s">
         <v>22</v>
       </c>
+      <c r="C14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
@@ -580,6 +592,12 @@
       <c r="B15" t="s">
         <v>23</v>
       </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -588,53 +606,95 @@
       <c r="B16" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B17" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B18" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B19" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B20" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B21" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B22" t="s">
         <v>23</v>
+      </c>
+      <c r="C22" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>